<commit_message>
feat: clean up Example project for a working demo
Remove test artifacts from Example project JSON:
- Drop TestScenario_missingParam (intentionally broken)
- Drop TestScenario2 (edge-case comma handling, steady state)
- Drop PopulationScenarioFromCSV (duplicate)
- Drop MissingParam and "Sheet, with comma" parameter groups
- Drop TestPopulation_noOnto (test variant)

Add proper demo content:
- Rename scenarios: Aciclovir_iv, Aciclovir_iv_female, Aciclovir_iv_population
- Rename individuals: Adult_male, Adult_female (new)
- Rename population: European_adults (50 individuals, 50% female)
- Descriptive plot titles and grid names
- Export configuration for Individual_diagnostics grid
- Fix typo "Aciclovri" → "Aciclovir"

Rename data file: TestProject_TimeValuesData → Aciclovir_TimeValuesData.
Regenerate all Excel files from updated JSON.
Update demo script, vignettes, and README to use new scenario names.
</commit_message>
<xml_diff>
--- a/inst/extdata/projects/Example/Configurations/Individuals.xlsx
+++ b/inst/extdata/projects/Example/Configurations/Individuals.xlsx
@@ -1,96 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub repositories\ESQlabs\esqlabsR\inst\extdata\examples\TestProject\Configurations\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FF58CB-4ADB-4D8E-AA1B-9DFAF4644EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7920" yWindow="5265" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="IndividualBiometrics" sheetId="1" r:id="rId1"/>
-    <sheet name="Indiv1" sheetId="2" r:id="rId2"/>
+    <sheet name="Renal" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
-  <si>
-    <t>IndividualId</t>
-  </si>
-  <si>
-    <t>Species</t>
-  </si>
-  <si>
-    <t>Population</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>Weight [kg]</t>
-  </si>
-  <si>
-    <t>Height [cm]</t>
-  </si>
-  <si>
-    <t>Age [year(s)]</t>
-  </si>
-  <si>
-    <t>Protein Ontogenies</t>
-  </si>
-  <si>
-    <t>Individual Parameter Sets</t>
-  </si>
-  <si>
-    <t>Indiv1</t>
-  </si>
-  <si>
-    <t>Human</t>
-  </si>
-  <si>
-    <t>European_ICRP_2002</t>
-  </si>
-  <si>
-    <t>MALE</t>
-  </si>
-  <si>
-    <t>CYP3A4:CYP3A4,CYP2D6:CYP2C8</t>
-  </si>
-  <si>
-    <t>Container Path</t>
-  </si>
-  <si>
-    <t>Parameter Name</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Units</t>
-  </si>
-  <si>
-    <t>Organism|Kidney</t>
-  </si>
-  <si>
-    <t>GFR</t>
-  </si>
-  <si>
-    <t>ml/min</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,21 +64,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -190,7 +108,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -224,7 +142,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -259,10 +176,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -435,62 +351,77 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.140625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>IndividualId</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Weight [kg]</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Height [cm]</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Age [year(s)]</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Protein Ontogenies</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Individual Parameter Sets</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Adult_male</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>European_ICRP_2002</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MALE</t>
+        </is>
       </c>
       <c r="E2">
         <v>73</v>
@@ -501,11 +432,56 @@
       <c r="G2">
         <v>30</v>
       </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>9</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>CYP3A4:CYP3A4</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Renal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Adult_female</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>European_ICRP_2002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FEMALE</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>60</v>
+      </c>
+      <c r="F3">
+        <v>165</v>
+      </c>
+      <c r="G3">
+        <v>28</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>CYP3A4:CYP3A4</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Renal</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -514,36 +490,50 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>17</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Container Path</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Parameter Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Organism|Kidney</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GFR</t>
+        </is>
       </c>
       <c r="C2">
         <v>90</v>
       </c>
-      <c r="D2" t="s">
-        <v>20</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ml/min</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>